<commit_message>
update README and Dataset
</commit_message>
<xml_diff>
--- a/code/Hist2Pheno_pkg/dataset/Hist2Pheno_Datasets.xlsx
+++ b/code/Hist2Pheno_pkg/dataset/Hist2Pheno_Datasets.xlsx
@@ -1352,13 +1352,13 @@
         <v>2</v>
       </c>
       <c r="L7" s="5" t="n">
-        <v>213403</v>
+        <v>175210</v>
       </c>
       <c r="M7" s="5" t="n">
-        <v>202495</v>
+        <v>175210</v>
       </c>
       <c r="N7" s="5" t="n">
-        <v>202483</v>
+        <v>175208</v>
       </c>
       <c r="O7" s="5" t="n">
         <v>1342478</v>
@@ -1367,20 +1367,20 @@
         <v>0</v>
       </c>
       <c r="Q7" s="5" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="R7" s="5" t="n">
         <v>16</v>
       </c>
       <c r="S7" s="5" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="T7" s="5" t="n">
         <v>5</v>
       </c>
       <c r="U7" s="4" t="inlineStr">
         <is>
-          <t>SN1–SN9; Rec GD/nonGD (sparse)</t>
+          <t>L12=SN1–SN9; Rec GD/nonGD (sparse); Mac_SEPP1 many-to-many L1</t>
         </is>
       </c>
       <c r="V7" s="5" t="n">
@@ -1418,7 +1418,7 @@
       </c>
       <c r="AC7" s="4" t="inlineStr">
         <is>
-          <t>Folder named CODEX for pipeline layout. GT_cells = 53,305 + 160,098 nuclei. GT_cells_on_HE = 46,699 + 155,796. StarDist_matched = 46,689 + 155,794. StarDist_all = 178,303 + 1,164,175. L12 copies L1. Train drops Unknown/LowQ. Original table Cell Type=17 counted a mixed Ini/Rec L2 union; canonical is 18 all / 16 train.</t>
+          <t>Folder named CODEX for pipeline layout; images are microscope H&amp;E + Visium HD nuclei. Heads: L2=subcluster (16), L12=spatial_niche SN1–SN9 (9), L1=cell_type (5). Drops Unknown/LowQ and SN LowQ/missing; trainable GT 37,371 Ini + 137,839 Rec (was 213,403 all-label nuclei). StarDist_matched 37,369 + 137,839. StarDist_all 178,303 + 1,164,175. Group CV is leave-one-replicate-out; when n_sections &lt; cv_k, best_mlp_gpu.pt is refit on all samples. Mac_SEPP1: Ini Vascular vs Rec Myeloid.</t>
         </is>
       </c>
     </row>
@@ -1539,7 +1539,7 @@
       </c>
       <c r="AC8" s="2" t="inlineStr">
         <is>
-          <t>GT_cells = supervised sheets 167,780 + 118,752 (original table 285,532 was 1k short). GT_cells_on_HE = 157,183 + 107,335. StarDist_matched = 146,878 + 98,190. StarDist_all = 252,179 + 245,840. Match drops Unlabeled + 3 red L2 (hybrids + Perivascular-Like) → 16/8/4 trainable. Leave-one-replicate-out CV.</t>
+          <t>GT_cells = supervised sheets 167,780 + 118,752. GT_cells_on_HE = 157,183 + 107,335. StarDist_matched = 146,878 + 98,190. StarDist_all = 252,179 + 245,840. Match drops Unlabeled + 3 red L2 (hybrids + Perivascular-Like) → 16/8/4 trainable. Group CV is leave-one-replicate-out; when n_sections &lt; cv_k, deployment weights (best_mlp_gpu.pt) are refit on all samples; OOF stays LORO. Notebook SKIP_POOLED_TRAIN=True loads that checkpoint.</t>
         </is>
       </c>
     </row>
@@ -1716,21 +1716,21 @@
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>GT nuclei (all labels)</t>
+          <t>GT nuclei (trainable)</t>
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>53305</v>
+        <v>37371</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>160098</v>
+        <v>137839</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>213403</v>
+        <v>175210</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Results/gbm_*_cell_info_HE_by_annotation.csv</t>
+          <t>Results/gbm_*_cell_info_HE_by_annotation.csv after Unknown/LowQ + SN LowQ drop</t>
         </is>
       </c>
     </row>
@@ -1741,17 +1741,17 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>46699</v>
+        <v>37371</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>155796</v>
+        <v>137839</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>202495</v>
+        <v>175210</v>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Cases/*/P*_cells_with_pixel.csv</t>
+          <t>Cases/*/P*_cells_with_pixel.csv (trainable)</t>
         </is>
       </c>
     </row>
@@ -1762,17 +1762,17 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>46689</v>
+        <v>37369</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>155794</v>
+        <v>137839</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>202483</v>
+        <v>175208</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>median 0.66 / 0.78 px</t>
+          <t>median still &lt; 1 px</t>
         </is>
       </c>
     </row>
@@ -1800,140 +1800,150 @@
     <row r="8" ht="28" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>L1 cell_type (all)</t>
+          <t>L1 cell_type (trainable)</t>
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>union 7</t>
-        </is>
+        <v>5</v>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>5</v>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>LowQ only in Ini</t>
+          <t>Tumor / Myeloid / Lymph / Oligo / Vascular</t>
         </is>
       </c>
     </row>
     <row r="9" ht="28" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>L1 trainable</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="C9" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="D9" s="5" t="n">
-        <v>5</v>
+          <t>L1 dropped</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Unknown, LowQ</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>excluded</t>
+        </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>drop Unknown, LowQ</t>
+          <t>not in hierarchy xlsx</t>
         </is>
       </c>
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>L2 subcluster (all)</t>
+          <t>L2 subcluster (trainable)</t>
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C10" s="3" t="n">
         <v>16</v>
       </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>union 18</t>
-        </is>
+      <c r="D10" s="2" t="n">
+        <v>16</v>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Ini lacks G1S/G2M/NPC-like; Rec lacks LowQ</t>
+          <t>Ini lacks G1S/G2M/NPC-like; Rec has all 16</t>
         </is>
       </c>
     </row>
     <row r="11" ht="28" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>L2 trainable</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="n">
-        <v>13</v>
-      </c>
-      <c r="C11" s="5" t="n">
-        <v>15</v>
-      </c>
-      <c r="D11" s="5" t="n">
-        <v>16</v>
+          <t>L2 dropped</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Unknown, LowQ</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>excluded</t>
+        </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>drop Unknown, LowQ; keep lowQ_vas</t>
+          <t>lowQ_vas kept</t>
         </is>
       </c>
     </row>
     <row r="12" ht="28" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>L12</t>
-        </is>
-      </c>
-      <c r="B12" s="2">
-        <f>L1</f>
-        <v/>
-      </c>
-      <c r="C12" s="2">
-        <f>L1</f>
-        <v/>
+          <t>L12 spatial_niche</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>SN1,2,5,6,8,9</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>SN1–SN7</t>
+        </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>copy of L1</t>
+          <t>SN1–SN9 (9)</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>no HCC-style third layer</t>
+          <t>L12 = spatial_niche; not a copy of L1. SN3/4/7 Rec-only; SN8/9 Ini-only</t>
         </is>
       </c>
     </row>
     <row r="13" ht="28" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>spatial_niche SN</t>
+          <t>L12 dropped</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>SN1–SN9 + LowQ</t>
+          <t>LowQ / missing</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>SN1–SN7 (no SN8/SN9)</t>
+          <t>LowQ / missing</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>SN1–SN9</t>
+          <t>excluded</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>max intersect_ratio 16 µm bin</t>
+          <t>filter_usable_gbm_sn</t>
         </is>
       </c>
     </row>
@@ -2049,7 +2059,7 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>2026-09-08. Completes the hand-made overview with verified counts from code/*/README.md, hierarchy Excel, palettes, and on-disk CSVs.</t>
+          <t>2026-09-09. GBM heads are subcluster (L2) / spatial_niche (L12) / cell_type (L1); Unknown/LowQ and SN LowQ dropped. Completes the overview with verified counts from code/*/README.md, hierarchy Excel, palettes, Results CSVs, and Cases match tables.</t>
         </is>
       </c>
     </row>
@@ -2169,7 +2179,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Hist2Pheno heads: fine / intermediate / coarse. GBM has only two biological layers, so L12 copies L1.</t>
+          <t>Hist2Pheno heads: fine / intermediate / coarse. GBM L2=subcluster, L12=spatial_niche (SN1–SN9), L1=cell_type (Tumor/Myeloid/Lymph/Oligo/Vascular). Not a copy of L1.</t>
         </is>
       </c>
     </row>
@@ -2220,7 +2230,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J198"/>
+  <dimension ref="A1:J210"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8844,12 +8854,12 @@
         </is>
       </c>
       <c r="H161" s="5" t="n">
-        <v>16459</v>
+        <v>12736</v>
       </c>
       <c r="I161" s="5" t="n">
-        <v>15241</v>
-      </c>
-      <c r="J161" s="4" t="inlineStr"/>
+        <v>12441</v>
+      </c>
+      <c r="J161" s="4" t="n"/>
     </row>
     <row r="162" ht="28" customHeight="1">
       <c r="A162" s="2" t="inlineStr">
@@ -8888,12 +8898,12 @@
         </is>
       </c>
       <c r="H162" s="3" t="n">
-        <v>5227</v>
+        <v>4735</v>
       </c>
       <c r="I162" s="3" t="n">
-        <v>25734</v>
-      </c>
-      <c r="J162" s="2" t="inlineStr"/>
+        <v>23677</v>
+      </c>
+      <c r="J162" s="2" t="n"/>
     </row>
     <row r="163" ht="28" customHeight="1">
       <c r="A163" s="4" t="inlineStr">
@@ -8932,12 +8942,12 @@
         </is>
       </c>
       <c r="H163" s="5" t="n">
-        <v>7392</v>
+        <v>6009</v>
       </c>
       <c r="I163" s="5" t="n">
-        <v>19607</v>
-      </c>
-      <c r="J163" s="4" t="inlineStr"/>
+        <v>17657</v>
+      </c>
+      <c r="J163" s="4" t="n"/>
     </row>
     <row r="164" ht="28" customHeight="1">
       <c r="A164" s="2" t="inlineStr">
@@ -8979,7 +8989,7 @@
         <v>0</v>
       </c>
       <c r="I164" s="3" t="n">
-        <v>21433</v>
+        <v>19453</v>
       </c>
       <c r="J164" s="2" t="inlineStr">
         <is>
@@ -9027,7 +9037,7 @@
         <v>0</v>
       </c>
       <c r="I165" s="5" t="n">
-        <v>17917</v>
+        <v>16142</v>
       </c>
       <c r="J165" s="4" t="inlineStr">
         <is>
@@ -9075,7 +9085,7 @@
         <v>0</v>
       </c>
       <c r="I166" s="3" t="n">
-        <v>11215</v>
+        <v>10059</v>
       </c>
       <c r="J166" s="2" t="inlineStr">
         <is>
@@ -9120,12 +9130,12 @@
         </is>
       </c>
       <c r="H167" s="5" t="n">
-        <v>4542</v>
+        <v>3801</v>
       </c>
       <c r="I167" s="5" t="n">
-        <v>12313</v>
-      </c>
-      <c r="J167" s="4" t="inlineStr"/>
+        <v>11026</v>
+      </c>
+      <c r="J167" s="4" t="n"/>
     </row>
     <row r="168" ht="28" customHeight="1">
       <c r="A168" s="2" t="inlineStr">
@@ -9164,12 +9174,12 @@
         </is>
       </c>
       <c r="H168" s="3" t="n">
-        <v>1893</v>
+        <v>1323</v>
       </c>
       <c r="I168" s="3" t="n">
-        <v>6280</v>
-      </c>
-      <c r="J168" s="2" t="inlineStr"/>
+        <v>5034</v>
+      </c>
+      <c r="J168" s="2" t="n"/>
     </row>
     <row r="169" ht="28" customHeight="1">
       <c r="A169" s="4" t="inlineStr">
@@ -9208,12 +9218,12 @@
         </is>
       </c>
       <c r="H169" s="5" t="n">
-        <v>3145</v>
+        <v>2405</v>
       </c>
       <c r="I169" s="5" t="n">
-        <v>1556</v>
-      </c>
-      <c r="J169" s="4" t="inlineStr"/>
+        <v>1311</v>
+      </c>
+      <c r="J169" s="4" t="n"/>
     </row>
     <row r="170" ht="28" customHeight="1">
       <c r="A170" s="2" t="inlineStr">
@@ -9252,14 +9262,14 @@
         </is>
       </c>
       <c r="H170" s="3" t="n">
-        <v>443</v>
+        <v>398</v>
       </c>
       <c r="I170" s="3" t="n">
-        <v>2309</v>
+        <v>1898</v>
       </c>
       <c r="J170" s="2" t="inlineStr">
         <is>
-          <t>Ini Vascular vs Rec Myeloid; hierarchy uses majority Myeloid</t>
+          <t>Ini Vascular vs Rec Myeloid; hierarchy majority Myeloid</t>
         </is>
       </c>
     </row>
@@ -9300,12 +9310,12 @@
         </is>
       </c>
       <c r="H171" s="5" t="n">
-        <v>1125</v>
+        <v>779</v>
       </c>
       <c r="I171" s="5" t="n">
-        <v>854</v>
-      </c>
-      <c r="J171" s="4" t="inlineStr"/>
+        <v>655</v>
+      </c>
+      <c r="J171" s="4" t="n"/>
     </row>
     <row r="172" ht="28" customHeight="1">
       <c r="A172" s="2" t="inlineStr">
@@ -9344,12 +9354,12 @@
         </is>
       </c>
       <c r="H172" s="3" t="n">
-        <v>2534</v>
+        <v>1997</v>
       </c>
       <c r="I172" s="3" t="n">
-        <v>8661</v>
-      </c>
-      <c r="J172" s="2" t="inlineStr"/>
+        <v>7607</v>
+      </c>
+      <c r="J172" s="2" t="n"/>
     </row>
     <row r="173" ht="28" customHeight="1">
       <c r="A173" s="4" t="inlineStr">
@@ -9388,12 +9398,12 @@
         </is>
       </c>
       <c r="H173" s="5" t="n">
-        <v>2484</v>
+        <v>1893</v>
       </c>
       <c r="I173" s="5" t="n">
-        <v>7413</v>
-      </c>
-      <c r="J173" s="4" t="inlineStr"/>
+        <v>6418</v>
+      </c>
+      <c r="J173" s="4" t="n"/>
     </row>
     <row r="174" ht="28" customHeight="1">
       <c r="A174" s="2" t="inlineStr">
@@ -9432,12 +9442,12 @@
         </is>
       </c>
       <c r="H174" s="3" t="n">
-        <v>727</v>
+        <v>664</v>
       </c>
       <c r="I174" s="3" t="n">
-        <v>2634</v>
-      </c>
-      <c r="J174" s="2" t="inlineStr"/>
+        <v>2332</v>
+      </c>
+      <c r="J174" s="2" t="n"/>
     </row>
     <row r="175" ht="28" customHeight="1">
       <c r="A175" s="4" t="inlineStr">
@@ -9476,12 +9486,12 @@
         </is>
       </c>
       <c r="H175" s="5" t="n">
-        <v>335</v>
+        <v>309</v>
       </c>
       <c r="I175" s="5" t="n">
-        <v>1371</v>
-      </c>
-      <c r="J175" s="4" t="inlineStr"/>
+        <v>1170</v>
+      </c>
+      <c r="J175" s="4" t="n"/>
     </row>
     <row r="176" ht="28" customHeight="1">
       <c r="A176" s="2" t="inlineStr">
@@ -9520,10 +9530,10 @@
         </is>
       </c>
       <c r="H176" s="3" t="n">
-        <v>393</v>
+        <v>322</v>
       </c>
       <c r="I176" s="3" t="n">
-        <v>1258</v>
+        <v>959</v>
       </c>
       <c r="J176" s="2" t="inlineStr">
         <is>
@@ -9544,38 +9554,34 @@
       </c>
       <c r="C177" s="4" t="inlineStr">
         <is>
-          <t>L2</t>
+          <t>L12</t>
         </is>
       </c>
       <c r="D177" s="4" t="inlineStr">
         <is>
-          <t>fine</t>
+          <t>intermediate</t>
         </is>
       </c>
       <c r="E177" s="4" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>SN1</t>
         </is>
       </c>
       <c r="F177" s="4" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G177" s="4" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G177" s="4" t="n"/>
       <c r="H177" s="5" t="n">
-        <v>5957</v>
+        <v>5394</v>
       </c>
       <c r="I177" s="5" t="n">
-        <v>4302</v>
+        <v>66732</v>
       </c>
       <c r="J177" s="4" t="inlineStr">
         <is>
-          <t>dropped</t>
+          <t>Ini+Rec; Rec-heavy</t>
         </is>
       </c>
     </row>
@@ -9592,65 +9598,61 @@
       </c>
       <c r="C178" s="2" t="inlineStr">
         <is>
-          <t>L2</t>
+          <t>L12</t>
         </is>
       </c>
       <c r="D178" s="2" t="inlineStr">
         <is>
-          <t>fine</t>
+          <t>intermediate</t>
         </is>
       </c>
       <c r="E178" s="2" t="inlineStr">
         <is>
-          <t>LowQ</t>
+          <t>SN2</t>
         </is>
       </c>
       <c r="F178" s="2" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G178" s="2" t="inlineStr">
-        <is>
-          <t>LowQ</t>
-        </is>
-      </c>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G178" s="2" t="n"/>
       <c r="H178" s="3" t="n">
-        <v>649</v>
+        <v>25215</v>
       </c>
       <c r="I178" s="3" t="n">
-        <v>0</v>
+        <v>27342</v>
       </c>
       <c r="J178" s="2" t="inlineStr">
         <is>
-          <t>Ini only; dropped</t>
+          <t>Ini-dominant</t>
         </is>
       </c>
     </row>
     <row r="179" ht="28" customHeight="1">
       <c r="A179" s="4" t="inlineStr">
         <is>
-          <t>xenium_brca</t>
+          <t>codex_gbm</t>
         </is>
       </c>
       <c r="B179" s="4" t="inlineStr">
         <is>
-          <t>BRCA</t>
+          <t>GBM</t>
         </is>
       </c>
       <c r="C179" s="4" t="inlineStr">
         <is>
-          <t>L2</t>
+          <t>L12</t>
         </is>
       </c>
       <c r="D179" s="4" t="inlineStr">
         <is>
-          <t>fine</t>
+          <t>intermediate</t>
         </is>
       </c>
       <c r="E179" s="4" t="inlineStr">
         <is>
-          <t>DCIS_1</t>
+          <t>SN3</t>
         </is>
       </c>
       <c r="F179" s="4" t="inlineStr">
@@ -9658,39 +9660,43 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G179" s="4" t="inlineStr">
-        <is>
-          <t>DCIS</t>
-        </is>
-      </c>
-      <c r="H179" s="4" t="n"/>
-      <c r="I179" s="4" t="n"/>
-      <c r="J179" s="4" t="inlineStr"/>
+      <c r="G179" s="4" t="n"/>
+      <c r="H179" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I179" s="4" t="n">
+        <v>17953</v>
+      </c>
+      <c r="J179" s="4" t="inlineStr">
+        <is>
+          <t>Rec only</t>
+        </is>
+      </c>
     </row>
     <row r="180" ht="28" customHeight="1">
       <c r="A180" s="2" t="inlineStr">
         <is>
-          <t>xenium_brca</t>
+          <t>codex_gbm</t>
         </is>
       </c>
       <c r="B180" s="2" t="inlineStr">
         <is>
-          <t>BRCA</t>
+          <t>GBM</t>
         </is>
       </c>
       <c r="C180" s="2" t="inlineStr">
         <is>
-          <t>L2</t>
+          <t>L12</t>
         </is>
       </c>
       <c r="D180" s="2" t="inlineStr">
         <is>
-          <t>fine</t>
+          <t>intermediate</t>
         </is>
       </c>
       <c r="E180" s="2" t="inlineStr">
         <is>
-          <t>DCIS_2</t>
+          <t>SN4</t>
         </is>
       </c>
       <c r="F180" s="2" t="inlineStr">
@@ -9698,39 +9704,43 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G180" s="2" t="inlineStr">
-        <is>
-          <t>DCIS</t>
-        </is>
-      </c>
-      <c r="H180" s="2" t="n"/>
-      <c r="I180" s="2" t="n"/>
-      <c r="J180" s="2" t="inlineStr"/>
+      <c r="G180" s="2" t="n"/>
+      <c r="H180" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I180" s="2" t="n">
+        <v>7433</v>
+      </c>
+      <c r="J180" s="2" t="inlineStr">
+        <is>
+          <t>Rec only</t>
+        </is>
+      </c>
     </row>
     <row r="181" ht="28" customHeight="1">
       <c r="A181" s="4" t="inlineStr">
         <is>
-          <t>xenium_brca</t>
+          <t>codex_gbm</t>
         </is>
       </c>
       <c r="B181" s="4" t="inlineStr">
         <is>
-          <t>BRCA</t>
+          <t>GBM</t>
         </is>
       </c>
       <c r="C181" s="4" t="inlineStr">
         <is>
-          <t>L2</t>
+          <t>L12</t>
         </is>
       </c>
       <c r="D181" s="4" t="inlineStr">
         <is>
-          <t>fine</t>
+          <t>intermediate</t>
         </is>
       </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
-          <t>Invasive_Tumor</t>
+          <t>SN5</t>
         </is>
       </c>
       <c r="F181" s="4" t="inlineStr">
@@ -9738,39 +9748,43 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G181" s="4" t="inlineStr">
-        <is>
-          <t>Invasive tumor</t>
-        </is>
-      </c>
-      <c r="H181" s="4" t="n"/>
-      <c r="I181" s="4" t="n"/>
-      <c r="J181" s="4" t="inlineStr"/>
+      <c r="G181" s="4" t="n"/>
+      <c r="H181" s="4" t="n">
+        <v>4594</v>
+      </c>
+      <c r="I181" s="4" t="n">
+        <v>13400</v>
+      </c>
+      <c r="J181" s="4" t="inlineStr">
+        <is>
+          <t>Ini+Rec</t>
+        </is>
+      </c>
     </row>
     <row r="182" ht="28" customHeight="1">
       <c r="A182" s="2" t="inlineStr">
         <is>
-          <t>xenium_brca</t>
+          <t>codex_gbm</t>
         </is>
       </c>
       <c r="B182" s="2" t="inlineStr">
         <is>
-          <t>BRCA</t>
+          <t>GBM</t>
         </is>
       </c>
       <c r="C182" s="2" t="inlineStr">
         <is>
-          <t>L2</t>
+          <t>L12</t>
         </is>
       </c>
       <c r="D182" s="2" t="inlineStr">
         <is>
-          <t>fine</t>
+          <t>intermediate</t>
         </is>
       </c>
       <c r="E182" s="2" t="inlineStr">
         <is>
-          <t>Prolif_Invasive_Tumor</t>
+          <t>SN6</t>
         </is>
       </c>
       <c r="F182" s="2" t="inlineStr">
@@ -9778,39 +9792,43 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G182" s="2" t="inlineStr">
-        <is>
-          <t>Invasive tumor</t>
-        </is>
-      </c>
-      <c r="H182" s="2" t="n"/>
-      <c r="I182" s="2" t="n"/>
-      <c r="J182" s="2" t="inlineStr"/>
+      <c r="G182" s="2" t="n"/>
+      <c r="H182" s="2" t="n">
+        <v>1040</v>
+      </c>
+      <c r="I182" s="2" t="n">
+        <v>3877</v>
+      </c>
+      <c r="J182" s="2" t="inlineStr">
+        <is>
+          <t>Ini+Rec</t>
+        </is>
+      </c>
     </row>
     <row r="183" ht="28" customHeight="1">
       <c r="A183" s="4" t="inlineStr">
         <is>
-          <t>xenium_brca</t>
+          <t>codex_gbm</t>
         </is>
       </c>
       <c r="B183" s="4" t="inlineStr">
         <is>
-          <t>BRCA</t>
+          <t>GBM</t>
         </is>
       </c>
       <c r="C183" s="4" t="inlineStr">
         <is>
-          <t>L2</t>
+          <t>L12</t>
         </is>
       </c>
       <c r="D183" s="4" t="inlineStr">
         <is>
-          <t>fine</t>
+          <t>intermediate</t>
         </is>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
-          <t>Myoepi_ACTA2+</t>
+          <t>SN7</t>
         </is>
       </c>
       <c r="F183" s="4" t="inlineStr">
@@ -9818,39 +9836,43 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G183" s="4" t="inlineStr">
-        <is>
-          <t>Myoepithelial</t>
-        </is>
-      </c>
-      <c r="H183" s="4" t="n"/>
-      <c r="I183" s="4" t="n"/>
-      <c r="J183" s="4" t="inlineStr"/>
+      <c r="G183" s="4" t="n"/>
+      <c r="H183" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I183" s="4" t="n">
+        <v>1102</v>
+      </c>
+      <c r="J183" s="4" t="inlineStr">
+        <is>
+          <t>Rec only</t>
+        </is>
+      </c>
     </row>
     <row r="184" ht="28" customHeight="1">
       <c r="A184" s="2" t="inlineStr">
         <is>
-          <t>xenium_brca</t>
+          <t>codex_gbm</t>
         </is>
       </c>
       <c r="B184" s="2" t="inlineStr">
         <is>
-          <t>BRCA</t>
+          <t>GBM</t>
         </is>
       </c>
       <c r="C184" s="2" t="inlineStr">
         <is>
-          <t>L2</t>
+          <t>L12</t>
         </is>
       </c>
       <c r="D184" s="2" t="inlineStr">
         <is>
-          <t>fine</t>
+          <t>intermediate</t>
         </is>
       </c>
       <c r="E184" s="2" t="inlineStr">
         <is>
-          <t>Myoepi_KRT15+</t>
+          <t>SN8</t>
         </is>
       </c>
       <c r="F184" s="2" t="inlineStr">
@@ -9858,83 +9880,87 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G184" s="2" t="inlineStr">
-        <is>
-          <t>Myoepithelial</t>
-        </is>
-      </c>
-      <c r="H184" s="2" t="n"/>
-      <c r="I184" s="2" t="n"/>
-      <c r="J184" s="2" t="inlineStr"/>
+      <c r="G184" s="2" t="n"/>
+      <c r="H184" s="2" t="n">
+        <v>973</v>
+      </c>
+      <c r="I184" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J184" s="2" t="inlineStr">
+        <is>
+          <t>Ini only</t>
+        </is>
+      </c>
     </row>
     <row r="185" ht="28" customHeight="1">
       <c r="A185" s="4" t="inlineStr">
         <is>
-          <t>xenium_brca</t>
+          <t>codex_gbm</t>
         </is>
       </c>
       <c r="B185" s="4" t="inlineStr">
         <is>
-          <t>BRCA</t>
+          <t>GBM</t>
         </is>
       </c>
       <c r="C185" s="4" t="inlineStr">
         <is>
-          <t>L2</t>
+          <t>L12</t>
         </is>
       </c>
       <c r="D185" s="4" t="inlineStr">
         <is>
-          <t>fine</t>
+          <t>intermediate</t>
         </is>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
-          <t>T_Cell_&amp;_Tumor_Hybrid</t>
+          <t>SN9</t>
         </is>
       </c>
       <c r="F185" s="4" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G185" s="4" t="inlineStr">
-        <is>
-          <t>Tumor–T-cell hybrid</t>
-        </is>
-      </c>
-      <c r="H185" s="4" t="n"/>
-      <c r="I185" s="4" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G185" s="4" t="n"/>
+      <c r="H185" s="4" t="n">
+        <v>155</v>
+      </c>
+      <c r="I185" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="J185" s="4" t="inlineStr">
         <is>
-          <t>dropped at match</t>
+          <t>Ini only</t>
         </is>
       </c>
     </row>
     <row r="186" ht="28" customHeight="1">
       <c r="A186" s="2" t="inlineStr">
         <is>
-          <t>xenium_brca</t>
+          <t>codex_gbm</t>
         </is>
       </c>
       <c r="B186" s="2" t="inlineStr">
         <is>
-          <t>BRCA</t>
+          <t>GBM</t>
         </is>
       </c>
       <c r="C186" s="2" t="inlineStr">
         <is>
-          <t>L2</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="D186" s="2" t="inlineStr">
         <is>
-          <t>fine</t>
+          <t>coarse</t>
         </is>
       </c>
       <c r="E186" s="2" t="inlineStr">
         <is>
-          <t>CD4+_T_Cells</t>
+          <t>Tumor</t>
         </is>
       </c>
       <c r="F186" s="2" t="inlineStr">
@@ -9942,39 +9968,43 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G186" s="2" t="inlineStr">
-        <is>
-          <t>T cells</t>
-        </is>
-      </c>
-      <c r="H186" s="2" t="n"/>
-      <c r="I186" s="2" t="n"/>
-      <c r="J186" s="2" t="inlineStr"/>
+      <c r="G186" s="2" t="n"/>
+      <c r="H186" s="2" t="n">
+        <v>23480</v>
+      </c>
+      <c r="I186" s="2" t="n">
+        <v>99429</v>
+      </c>
+      <c r="J186" s="2" t="inlineStr">
+        <is>
+          <t>cell_type</t>
+        </is>
+      </c>
     </row>
     <row r="187" ht="28" customHeight="1">
       <c r="A187" s="4" t="inlineStr">
         <is>
-          <t>xenium_brca</t>
+          <t>codex_gbm</t>
         </is>
       </c>
       <c r="B187" s="4" t="inlineStr">
         <is>
-          <t>BRCA</t>
+          <t>GBM</t>
         </is>
       </c>
       <c r="C187" s="4" t="inlineStr">
         <is>
-          <t>L2</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="D187" s="4" t="inlineStr">
         <is>
-          <t>fine</t>
+          <t>coarse</t>
         </is>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
-          <t>CD8+_T_Cells</t>
+          <t>Myeloid</t>
         </is>
       </c>
       <c r="F187" s="4" t="inlineStr">
@@ -9982,39 +10012,43 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G187" s="4" t="inlineStr">
-        <is>
-          <t>T cells</t>
-        </is>
-      </c>
-      <c r="H187" s="4" t="n"/>
-      <c r="I187" s="4" t="n"/>
-      <c r="J187" s="4" t="inlineStr"/>
+      <c r="G187" s="4" t="n"/>
+      <c r="H187" s="4" t="n">
+        <v>7529</v>
+      </c>
+      <c r="I187" s="4" t="n">
+        <v>19269</v>
+      </c>
+      <c r="J187" s="4" t="inlineStr">
+        <is>
+          <t>cell_type</t>
+        </is>
+      </c>
     </row>
     <row r="188" ht="28" customHeight="1">
       <c r="A188" s="2" t="inlineStr">
         <is>
-          <t>xenium_brca</t>
+          <t>codex_gbm</t>
         </is>
       </c>
       <c r="B188" s="2" t="inlineStr">
         <is>
-          <t>BRCA</t>
+          <t>GBM</t>
         </is>
       </c>
       <c r="C188" s="2" t="inlineStr">
         <is>
-          <t>L2</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="D188" s="2" t="inlineStr">
         <is>
-          <t>fine</t>
+          <t>coarse</t>
         </is>
       </c>
       <c r="E188" s="2" t="inlineStr">
         <is>
-          <t>B_Cells</t>
+          <t>Lymph</t>
         </is>
       </c>
       <c r="F188" s="2" t="inlineStr">
@@ -10022,39 +10056,43 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G188" s="2" t="inlineStr">
-        <is>
-          <t>B cells</t>
-        </is>
-      </c>
-      <c r="H188" s="2" t="n"/>
-      <c r="I188" s="2" t="n"/>
-      <c r="J188" s="2" t="inlineStr"/>
+      <c r="G188" s="2" t="n"/>
+      <c r="H188" s="2" t="n">
+        <v>779</v>
+      </c>
+      <c r="I188" s="2" t="n">
+        <v>655</v>
+      </c>
+      <c r="J188" s="2" t="inlineStr">
+        <is>
+          <t>cell_type</t>
+        </is>
+      </c>
     </row>
     <row r="189" ht="28" customHeight="1">
       <c r="A189" s="4" t="inlineStr">
         <is>
-          <t>xenium_brca</t>
+          <t>codex_gbm</t>
         </is>
       </c>
       <c r="B189" s="4" t="inlineStr">
         <is>
-          <t>BRCA</t>
+          <t>GBM</t>
         </is>
       </c>
       <c r="C189" s="4" t="inlineStr">
         <is>
-          <t>L2</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="D189" s="4" t="inlineStr">
         <is>
-          <t>fine</t>
+          <t>coarse</t>
         </is>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
-          <t>Macrophages_1</t>
+          <t>Oligo</t>
         </is>
       </c>
       <c r="F189" s="4" t="inlineStr">
@@ -10062,39 +10100,43 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G189" s="4" t="inlineStr">
-        <is>
-          <t>Myeloid</t>
-        </is>
-      </c>
-      <c r="H189" s="4" t="n"/>
-      <c r="I189" s="4" t="n"/>
-      <c r="J189" s="4" t="inlineStr"/>
+      <c r="G189" s="4" t="n"/>
+      <c r="H189" s="4" t="n">
+        <v>1997</v>
+      </c>
+      <c r="I189" s="4" t="n">
+        <v>7607</v>
+      </c>
+      <c r="J189" s="4" t="inlineStr">
+        <is>
+          <t>cell_type</t>
+        </is>
+      </c>
     </row>
     <row r="190" ht="28" customHeight="1">
       <c r="A190" s="2" t="inlineStr">
         <is>
-          <t>xenium_brca</t>
+          <t>codex_gbm</t>
         </is>
       </c>
       <c r="B190" s="2" t="inlineStr">
         <is>
-          <t>BRCA</t>
+          <t>GBM</t>
         </is>
       </c>
       <c r="C190" s="2" t="inlineStr">
         <is>
-          <t>L2</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="D190" s="2" t="inlineStr">
         <is>
-          <t>fine</t>
+          <t>coarse</t>
         </is>
       </c>
       <c r="E190" s="2" t="inlineStr">
         <is>
-          <t>Macrophages_2</t>
+          <t>Vascular</t>
         </is>
       </c>
       <c r="F190" s="2" t="inlineStr">
@@ -10102,14 +10144,18 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G190" s="2" t="inlineStr">
-        <is>
-          <t>Myeloid</t>
-        </is>
-      </c>
-      <c r="H190" s="2" t="n"/>
-      <c r="I190" s="2" t="n"/>
-      <c r="J190" s="2" t="inlineStr"/>
+      <c r="G190" s="2" t="n"/>
+      <c r="H190" s="2" t="n">
+        <v>3586</v>
+      </c>
+      <c r="I190" s="2" t="n">
+        <v>10879</v>
+      </c>
+      <c r="J190" s="2" t="inlineStr">
+        <is>
+          <t>cell_type</t>
+        </is>
+      </c>
     </row>
     <row r="191" ht="28" customHeight="1">
       <c r="A191" s="4" t="inlineStr">
@@ -10134,7 +10180,7 @@
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
-          <t>IRF7+_DCs</t>
+          <t>DCIS_1</t>
         </is>
       </c>
       <c r="F191" s="4" t="inlineStr">
@@ -10144,12 +10190,12 @@
       </c>
       <c r="G191" s="4" t="inlineStr">
         <is>
-          <t>Myeloid</t>
+          <t>DCIS</t>
         </is>
       </c>
       <c r="H191" s="4" t="n"/>
       <c r="I191" s="4" t="n"/>
-      <c r="J191" s="4" t="inlineStr"/>
+      <c r="J191" s="4" t="n"/>
     </row>
     <row r="192" ht="28" customHeight="1">
       <c r="A192" s="2" t="inlineStr">
@@ -10174,7 +10220,7 @@
       </c>
       <c r="E192" s="2" t="inlineStr">
         <is>
-          <t>LAMP3+_DCs</t>
+          <t>DCIS_2</t>
         </is>
       </c>
       <c r="F192" s="2" t="inlineStr">
@@ -10184,12 +10230,12 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>Myeloid</t>
+          <t>DCIS</t>
         </is>
       </c>
       <c r="H192" s="2" t="n"/>
       <c r="I192" s="2" t="n"/>
-      <c r="J192" s="2" t="inlineStr"/>
+      <c r="J192" s="2" t="n"/>
     </row>
     <row r="193" ht="28" customHeight="1">
       <c r="A193" s="4" t="inlineStr">
@@ -10214,7 +10260,7 @@
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
-          <t>Mast_Cells</t>
+          <t>Invasive_Tumor</t>
         </is>
       </c>
       <c r="F193" s="4" t="inlineStr">
@@ -10224,12 +10270,12 @@
       </c>
       <c r="G193" s="4" t="inlineStr">
         <is>
-          <t>Myeloid</t>
+          <t>Invasive tumor</t>
         </is>
       </c>
       <c r="H193" s="4" t="n"/>
       <c r="I193" s="4" t="n"/>
-      <c r="J193" s="4" t="inlineStr"/>
+      <c r="J193" s="4" t="n"/>
     </row>
     <row r="194" ht="28" customHeight="1">
       <c r="A194" s="2" t="inlineStr">
@@ -10254,26 +10300,22 @@
       </c>
       <c r="E194" s="2" t="inlineStr">
         <is>
-          <t>Stromal_&amp;_T_Cell_Hybrid</t>
+          <t>Prolif_Invasive_Tumor</t>
         </is>
       </c>
       <c r="F194" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="G194" s="2" t="inlineStr">
         <is>
-          <t>Stromal–T-cell hybrid</t>
+          <t>Invasive tumor</t>
         </is>
       </c>
       <c r="H194" s="2" t="n"/>
       <c r="I194" s="2" t="n"/>
-      <c r="J194" s="2" t="inlineStr">
-        <is>
-          <t>dropped at match</t>
-        </is>
-      </c>
+      <c r="J194" s="2" t="n"/>
     </row>
     <row r="195" ht="28" customHeight="1">
       <c r="A195" s="4" t="inlineStr">
@@ -10298,7 +10340,7 @@
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
-          <t>Stromal</t>
+          <t>Myoepi_ACTA2+</t>
         </is>
       </c>
       <c r="F195" s="4" t="inlineStr">
@@ -10308,12 +10350,12 @@
       </c>
       <c r="G195" s="4" t="inlineStr">
         <is>
-          <t>Stromal</t>
+          <t>Myoepithelial</t>
         </is>
       </c>
       <c r="H195" s="4" t="n"/>
       <c r="I195" s="4" t="n"/>
-      <c r="J195" s="4" t="inlineStr"/>
+      <c r="J195" s="4" t="n"/>
     </row>
     <row r="196" ht="28" customHeight="1">
       <c r="A196" s="2" t="inlineStr">
@@ -10338,7 +10380,7 @@
       </c>
       <c r="E196" s="2" t="inlineStr">
         <is>
-          <t>Endothelial</t>
+          <t>Myoepi_KRT15+</t>
         </is>
       </c>
       <c r="F196" s="2" t="inlineStr">
@@ -10348,12 +10390,12 @@
       </c>
       <c r="G196" s="2" t="inlineStr">
         <is>
-          <t>Endothelial</t>
+          <t>Myoepithelial</t>
         </is>
       </c>
       <c r="H196" s="2" t="n"/>
       <c r="I196" s="2" t="n"/>
-      <c r="J196" s="2" t="inlineStr"/>
+      <c r="J196" s="2" t="n"/>
     </row>
     <row r="197" ht="28" customHeight="1">
       <c r="A197" s="4" t="inlineStr">
@@ -10378,7 +10420,7 @@
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
-          <t>Perivascular-Like</t>
+          <t>T_Cell_&amp;_Tumor_Hybrid</t>
         </is>
       </c>
       <c r="F197" s="4" t="inlineStr">
@@ -10388,7 +10430,7 @@
       </c>
       <c r="G197" s="4" t="inlineStr">
         <is>
-          <t>Perivascular</t>
+          <t>Tumor–T-cell hybrid</t>
         </is>
       </c>
       <c r="H197" s="4" t="n"/>
@@ -10422,18 +10464,472 @@
       </c>
       <c r="E198" s="2" t="inlineStr">
         <is>
-          <t>Unlabeled</t>
+          <t>CD4+_T_Cells</t>
         </is>
       </c>
       <c r="F198" s="2" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G198" s="2" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G198" s="2" t="inlineStr">
+        <is>
+          <t>T cells</t>
+        </is>
+      </c>
       <c r="H198" s="2" t="n"/>
       <c r="I198" s="2" t="n"/>
-      <c r="J198" s="2" t="inlineStr">
+      <c r="J198" s="2" t="n"/>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>xenium_brca</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>BRCA</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>fine</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>CD8+_T_Cells</t>
+        </is>
+      </c>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G199" t="inlineStr">
+        <is>
+          <t>T cells</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>xenium_brca</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>BRCA</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>fine</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>B_Cells</t>
+        </is>
+      </c>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G200" t="inlineStr">
+        <is>
+          <t>B cells</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>xenium_brca</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>BRCA</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>fine</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>Macrophages_1</t>
+        </is>
+      </c>
+      <c r="F201" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G201" t="inlineStr">
+        <is>
+          <t>Myeloid</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>xenium_brca</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>BRCA</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>fine</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>Macrophages_2</t>
+        </is>
+      </c>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G202" t="inlineStr">
+        <is>
+          <t>Myeloid</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>xenium_brca</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>BRCA</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>fine</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>IRF7+_DCs</t>
+        </is>
+      </c>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G203" t="inlineStr">
+        <is>
+          <t>Myeloid</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>xenium_brca</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>BRCA</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>fine</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>LAMP3+_DCs</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G204" t="inlineStr">
+        <is>
+          <t>Myeloid</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>xenium_brca</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>BRCA</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>fine</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>Mast_Cells</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G205" t="inlineStr">
+        <is>
+          <t>Myeloid</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>xenium_brca</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>BRCA</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>fine</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>Stromal_&amp;_T_Cell_Hybrid</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G206" t="inlineStr">
+        <is>
+          <t>Stromal–T-cell hybrid</t>
+        </is>
+      </c>
+      <c r="J206" t="inlineStr">
+        <is>
+          <t>dropped at match</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>xenium_brca</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>BRCA</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>fine</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>Stromal</t>
+        </is>
+      </c>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G207" t="inlineStr">
+        <is>
+          <t>Stromal</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>xenium_brca</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>BRCA</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>fine</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>Endothelial</t>
+        </is>
+      </c>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G208" t="inlineStr">
+        <is>
+          <t>Endothelial</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>xenium_brca</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>BRCA</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>fine</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>Perivascular-Like</t>
+        </is>
+      </c>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G209" t="inlineStr">
+        <is>
+          <t>Perivascular</t>
+        </is>
+      </c>
+      <c r="J209" t="inlineStr">
+        <is>
+          <t>dropped at match</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>xenium_brca</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>BRCA</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>fine</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>Unlabeled</t>
+        </is>
+      </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="J210" t="inlineStr">
         <is>
           <t>dropped at match</t>
         </is>

</xml_diff>

<commit_message>
update pancancer cell label
</commit_message>
<xml_diff>
--- a/code/Hist2Pheno_pkg/dataset/Hist2Pheno_Datasets.xlsx
+++ b/code/Hist2Pheno_pkg/dataset/Hist2Pheno_Datasets.xlsx
@@ -12,22 +12,24 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hierarchy" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Xenium_lung" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Xenium_brca" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CODEX_hcc" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CODEX_escc" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CODEX_pdac" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CODEX_gist" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CODEX_gbm" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Xenium_crc" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CODEX_hcc" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CODEX_escc" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CODEX_pdac" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CODEX_gist" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CODEX_gbm" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Datasets'!$A$1:$AC$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Datasets'!$A$1:$AC$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Hierarchy'!$A$1:$J$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Xenium_lung'!$A$1:$P$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Xenium_brca'!$A$1:$M$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'CODEX_hcc'!$A$1:$M$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'CODEX_escc'!$A$1:$M$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'CODEX_pdac'!$A$1:$G$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'CODEX_gist'!$A$1:$G$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'CODEX_gbm'!$A$1:$E$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Xenium_crc'!$A$1:$M$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'CODEX_hcc'!$A$1:$M$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'CODEX_escc'!$A$1:$M$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'CODEX_pdac'!$A$1:$G$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'CODEX_gist'!$A$1:$G$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'CODEX_gbm'!$A$1:$E$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -543,7 +545,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC9"/>
+  <dimension ref="A1:AC10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1543,73 +1545,194 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="36" customHeight="1">
-      <c r="A9" s="6" t="inlineStr"/>
-      <c r="B9" s="6" t="inlineStr">
+    <row r="9" ht="28" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Xenium</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Colorectal carcinoma (Visium HD + Xenium)</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>结直肠癌</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>xenium_crc</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>code/Xenium_crc/</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>data/Xemium/CRC/ + data/VisiumHD/CRC/</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Xenium In Situ + Visium HD 8 µm RCTD (Oliveira FFPE CRC)</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="J9" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="K9" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="L9" s="3" t="n">
+        <v>364539</v>
+      </c>
+      <c r="M9" s="3" t="n">
+        <v>364539</v>
+      </c>
+      <c r="N9" s="3" t="n">
+        <v>263361</v>
+      </c>
+      <c r="O9" s="3" t="n">
+        <v>3112263</v>
+      </c>
+      <c r="P9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="3" t="n">
+        <v>39</v>
+      </c>
+      <c r="R9" s="3" t="n">
+        <v>38</v>
+      </c>
+      <c r="S9" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="T9" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="U9" s="2" t="inlineStr">
+        <is>
+          <t>L12=Flex 9-class Level1 (Neuronal folded into Stromal L1)</t>
+        </is>
+      </c>
+      <c r="V9" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="W9" s="2" t="inlineStr">
+        <is>
+          <t>train</t>
+        </is>
+      </c>
+      <c r="X9" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Y9" s="2" t="inlineStr">
+        <is>
+          <t>P1 vs P2 (P5 HE only; labels not transferred yet)</t>
+        </is>
+      </c>
+      <c r="Z9" s="2" t="inlineStr">
+        <is>
+          <t>Oliveira MF, Romero JP, Chung M, et al. High-definition spatial transcriptomic profiling of immune cell populations in colorectal cancer. Nat Genet 57, 1512–1523 (2025).</t>
+        </is>
+      </c>
+      <c r="AA9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.nature.com/articles/s41588-025-02193-3</t>
+        </is>
+      </c>
+      <c r="AB9" s="2" t="inlineStr">
+        <is>
+          <t>GSE280318; 10x Visium HD Human CRC</t>
+        </is>
+      </c>
+      <c r="AC9" s="2" t="inlineStr">
+        <is>
+          <t>Labels = Visium HD RCTD DeconvolutionLabel1 transferred onto Xenium cells (singlet only), not native Xenium GT. GT_cells = P1_CRC + P2_CRC annotation sheets 154,760 + 209,779 = 364,539 (same as Cases with_pixel). StarDist_matched = 96,858 + 166,503 = 263,361. StarDist_all P1+P2 = 1,594,379 + 1,517,884 = 3,112,263 (P5 StarDist missing). L2_all 39 = 38 Flex Level2 + Unlabeled; L2_train 38. L12_train 9 Flex Level1; L1_train 4 coarse. P5: HE OME + alignment CSV present; no annotation sheet / Cases / StarDist yet. UNI --scale ≈ 0.548 (0.274 µm/px). Group CV leave-one-patient-out when n_sections &lt; cv_k.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr"/>
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>ALL</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>Hist2Pheno cohorts</t>
         </is>
       </c>
-      <c r="D9" s="6" t="inlineStr">
+      <c r="D10" s="6" t="inlineStr">
         <is>
           <t>合计</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr"/>
-      <c r="F9" s="6" t="inlineStr"/>
-      <c r="G9" s="6" t="inlineStr"/>
-      <c r="H9" s="6" t="inlineStr"/>
-      <c r="I9" s="7">
-        <f>SUM(I2:I8)</f>
+      <c r="E10" s="6" t="inlineStr"/>
+      <c r="F10" s="6" t="inlineStr"/>
+      <c r="G10" s="6" t="inlineStr"/>
+      <c r="H10" s="6" t="inlineStr"/>
+      <c r="I10" s="7">
+        <f>SUM(I2:I9)</f>
         <v/>
       </c>
-      <c r="J9" s="7">
-        <f>SUM(J2:J8)</f>
+      <c r="J10" s="7">
+        <f>SUM(J2:J9)</f>
         <v/>
       </c>
-      <c r="K9" s="7">
-        <f>SUM(K2:K8)</f>
+      <c r="K10" s="7">
+        <f>SUM(K2:K9)</f>
         <v/>
       </c>
-      <c r="L9" s="7">
-        <f>SUM(L2:L8)</f>
+      <c r="L10" s="7">
+        <f>SUM(L2:L9)</f>
         <v/>
       </c>
-      <c r="M9" s="7">
-        <f>SUM(M2:M8)</f>
+      <c r="M10" s="7">
+        <f>SUM(M2:M9)</f>
         <v/>
       </c>
-      <c r="N9" s="6" t="n"/>
-      <c r="O9" s="6" t="n"/>
-      <c r="P9" s="7">
-        <f>SUM(P2:P8)</f>
+      <c r="N10" s="6" t="n"/>
+      <c r="O10" s="6" t="n"/>
+      <c r="P10" s="7">
+        <f>SUM(P2:P9)</f>
         <v/>
       </c>
-      <c r="Q9" s="6" t="inlineStr"/>
-      <c r="R9" s="6" t="inlineStr"/>
-      <c r="S9" s="6" t="inlineStr"/>
-      <c r="T9" s="6" t="inlineStr"/>
-      <c r="U9" s="6" t="inlineStr"/>
-      <c r="V9" s="6" t="inlineStr"/>
-      <c r="W9" s="6" t="inlineStr"/>
-      <c r="X9" s="6" t="inlineStr"/>
-      <c r="Y9" s="6" t="inlineStr"/>
-      <c r="Z9" s="6" t="inlineStr"/>
-      <c r="AA9" s="6" t="inlineStr"/>
-      <c r="AB9" s="6" t="inlineStr"/>
-      <c r="AC9" s="6" t="inlineStr">
+      <c r="Q10" s="6" t="inlineStr"/>
+      <c r="R10" s="6" t="inlineStr"/>
+      <c r="S10" s="6" t="inlineStr"/>
+      <c r="T10" s="6" t="inlineStr"/>
+      <c r="U10" s="6" t="inlineStr"/>
+      <c r="V10" s="6" t="inlineStr"/>
+      <c r="W10" s="6" t="inlineStr"/>
+      <c r="X10" s="6" t="inlineStr"/>
+      <c r="Y10" s="6" t="inlineStr"/>
+      <c r="Z10" s="6" t="inlineStr"/>
+      <c r="AA10" s="6" t="inlineStr"/>
+      <c r="AB10" s="6" t="inlineStr"/>
+      <c r="AC10" s="6" t="inlineStr">
         <is>
           <t>Sums skip blank StarDist columns. GT_cells mixes slightly different definitions — see Legend.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AC8"/>
+  <autoFilter ref="A1:AC9"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA3" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA4" r:id="rId2"/>
@@ -1621,6 +1744,187 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="55" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>coverslip</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>All_cores</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Annotated_cores</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Unlabeled_cores</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>GT_cells</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>L2_train</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>c009</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>160</v>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>160</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>GIST TMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>c011</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="n">
+        <v>197</v>
+      </c>
+      <c r="C3" s="5" t="n">
+        <v>197</v>
+      </c>
+      <c r="D3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="4" t="n"/>
+      <c r="F3" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>GIST TMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>c013</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>193</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>193</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>GIST TMA; demo Charvill-94_c013_v001_r001_reg002</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="28" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>All GIST</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>550</v>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>550</v>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>1785460</v>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>GT_cells from original overview (no Incomplete_Cases)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>L2 (11 train + Other): Epithelial cells, Fibroblasts, Stromal cells, Helper T cells, Tregs, T cells, Monocytes, Neutrophils, DCs, B cells, Endothelial cells, Other</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>L12/L1 same 6/4 structure as PDAC. Clinical recodes: site, size, mitotic, mutation, risk, primary, tma_block. StarDist: StarDist_Segment_gist/</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G1"/>
+  <mergeCells count="2">
+    <mergeCell ref="A8:G8"/>
+    <mergeCell ref="A7:G7"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2059,7 +2363,7 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>2026-09-09. GBM heads are subcluster (L2) / spatial_niche (L12) / cell_type (L1); Unknown/LowQ and SN LowQ dropped. Completes the overview with verified counts from code/*/README.md, hierarchy Excel, palettes, Results CSVs, and Cases match tables.</t>
+          <t>2026-09-15. Added Xenium CRC (Oliveira Nat Genet 2025; GSE280318): transferred Visium HD RCTD Label1, P1+P2 labeled / P5 HE only. GBM heads remain subcluster / spatial_niche / cell_type.</t>
         </is>
       </c>
     </row>
@@ -2230,7 +2534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J210"/>
+  <dimension ref="A1:J262"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -10932,6 +11236,2261 @@
       <c r="J210" t="inlineStr">
         <is>
           <t>dropped at match</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>xenium_crc</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>fine</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>Tumor I</t>
+        </is>
+      </c>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G211" t="inlineStr">
+        <is>
+          <t>Tumor</t>
+        </is>
+      </c>
+      <c r="H211" t="n">
+        <v>49</v>
+      </c>
+      <c r="I211" t="n">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>xenium_crc</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>fine</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>Tumor II</t>
+        </is>
+      </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G212" t="inlineStr">
+        <is>
+          <t>Tumor</t>
+        </is>
+      </c>
+      <c r="H212" t="n">
+        <v>80223</v>
+      </c>
+      <c r="I212" t="n">
+        <v>585</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>xenium_crc</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>fine</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>Tumor III</t>
+        </is>
+      </c>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G213" t="inlineStr">
+        <is>
+          <t>Tumor</t>
+        </is>
+      </c>
+      <c r="H213" t="n">
+        <v>436</v>
+      </c>
+      <c r="I213" t="n">
+        <v>146993</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>xenium_crc</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>fine</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>Tumor IV</t>
+        </is>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G214" t="inlineStr">
+        <is>
+          <t>Tumor</t>
+        </is>
+      </c>
+      <c r="H214" t="n">
+        <v>22</v>
+      </c>
+      <c r="I214" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>xenium_crc</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>fine</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>Tumor V</t>
+        </is>
+      </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G215" t="inlineStr">
+        <is>
+          <t>Tumor</t>
+        </is>
+      </c>
+      <c r="H215" t="n">
+        <v>751</v>
+      </c>
+      <c r="I215" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>xenium_crc</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>fine</t>
+        </is>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>Enterocyte</t>
+        </is>
+      </c>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G216" t="inlineStr">
+        <is>
+          <t>Intestinal Epithelial</t>
+        </is>
+      </c>
+      <c r="H216" t="n">
+        <v>2978</v>
+      </c>
+      <c r="I216" t="n">
+        <v>4808</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>xenium_crc</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>fine</t>
+        </is>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>Goblet</t>
+        </is>
+      </c>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G217" t="inlineStr">
+        <is>
+          <t>Intestinal Epithelial</t>
+        </is>
+      </c>
+      <c r="H217" t="n">
+        <v>19950</v>
+      </c>
+      <c r="I217" t="n">
+        <v>17397</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>xenium_crc</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>fine</t>
+        </is>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>Adipocyte</t>
+        </is>
+      </c>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G218" t="inlineStr">
+        <is>
+          <t>Fibroblast</t>
+        </is>
+      </c>
+      <c r="H218" t="n">
+        <v>6</v>
+      </c>
+      <c r="I218" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>xenium_crc</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>fine</t>
+        </is>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>CAF</t>
+        </is>
+      </c>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G219" t="inlineStr">
+        <is>
+          <t>Fibroblast</t>
+        </is>
+      </c>
+      <c r="H219" t="n">
+        <v>14343</v>
+      </c>
+      <c r="I219" t="n">
+        <v>15622</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>xenium_crc</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>fine</t>
+        </is>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>Fibroblast</t>
+        </is>
+      </c>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G220" t="inlineStr">
+        <is>
+          <t>Fibroblast</t>
+        </is>
+      </c>
+      <c r="H220" t="n">
+        <v>1725</v>
+      </c>
+      <c r="I220" t="n">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>xenium_crc</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>fine</t>
+        </is>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>Myofibroblast</t>
+        </is>
+      </c>
+      <c r="F221" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G221" t="inlineStr">
+        <is>
+          <t>Fibroblast</t>
+        </is>
+      </c>
+      <c r="H221" t="n">
+        <v>1710</v>
+      </c>
+      <c r="I221" t="n">
+        <v>1466</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>xenium_crc</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>fine</t>
+        </is>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>Pericytes</t>
+        </is>
+      </c>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G222" t="inlineStr">
+        <is>
+          <t>Fibroblast</t>
+        </is>
+      </c>
+      <c r="H222" t="n">
+        <v>2113</v>
+      </c>
+      <c r="I222" t="n">
+        <v>1427</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>xenium_crc</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>fine</t>
+        </is>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>Proliferating Fibroblast</t>
+        </is>
+      </c>
+      <c r="F223" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G223" t="inlineStr">
+        <is>
+          <t>Fibroblast</t>
+        </is>
+      </c>
+      <c r="H223" t="n">
+        <v>800</v>
+      </c>
+      <c r="I223" t="n">
+        <v>1005</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>xenium_crc</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>fine</t>
+        </is>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>Vascular Fibroblast</t>
+        </is>
+      </c>
+      <c r="F224" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G224" t="inlineStr">
+        <is>
+          <t>Fibroblast</t>
+        </is>
+      </c>
+      <c r="H224" t="n">
+        <v>1</v>
+      </c>
+      <c r="I224" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>xenium_crc</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>fine</t>
+        </is>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>Epithelial</t>
+        </is>
+      </c>
+      <c r="F225" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G225" t="inlineStr">
+        <is>
+          <t>Smooth Muscle</t>
+        </is>
+      </c>
+      <c r="H225" t="n">
+        <v>96</v>
+      </c>
+      <c r="I225" t="n">
+        <v>63</v>
+      </c>
+      <c r="J225" t="inlineStr">
+        <is>
+          <t>Flex parent=Smooth Muscle, not intestinal epithelium</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>xenium_crc</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>fine</t>
+        </is>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>SM Stress Response</t>
+        </is>
+      </c>
+      <c r="F226" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G226" t="inlineStr">
+        <is>
+          <t>Smooth Muscle</t>
+        </is>
+      </c>
+      <c r="H226" t="n">
+        <v>2</v>
+      </c>
+      <c r="I226" t="n">
+        <v>0</v>
+      </c>
+      <c r="J226" t="inlineStr">
+        <is>
+          <t>absent in P2 transferred singlets</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>xenium_crc</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>fine</t>
+        </is>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>Smooth Muscle</t>
+        </is>
+      </c>
+      <c r="F227" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G227" t="inlineStr">
+        <is>
+          <t>Smooth Muscle</t>
+        </is>
+      </c>
+      <c r="H227" t="n">
+        <v>78</v>
+      </c>
+      <c r="I227" t="n">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>xenium_crc</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>fine</t>
+        </is>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>Unknown III (SM)</t>
+        </is>
+      </c>
+      <c r="F228" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G228" t="inlineStr">
+        <is>
+          <t>Smooth Muscle</t>
+        </is>
+      </c>
+      <c r="H228" t="n">
+        <v>208</v>
+      </c>
+      <c r="I228" t="n">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>xenium_crc</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>fine</t>
+        </is>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>vSM</t>
+        </is>
+      </c>
+      <c r="F229" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G229" t="inlineStr">
+        <is>
+          <t>Smooth Muscle</t>
+        </is>
+      </c>
+      <c r="H229" t="n">
+        <v>1717</v>
+      </c>
+      <c r="I229" t="n">
+        <v>3813</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>xenium_crc</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>fine</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>Enteric Glial</t>
+        </is>
+      </c>
+      <c r="F230" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G230" t="inlineStr">
+        <is>
+          <t>Neuronal</t>
+        </is>
+      </c>
+      <c r="H230" t="n">
+        <v>322</v>
+      </c>
+      <c r="I230" t="n">
+        <v>135</v>
+      </c>
+      <c r="J230" t="inlineStr">
+        <is>
+          <t>pan-cancer v1 → Neural</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>xenium_crc</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>fine</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>Neuroendocrine</t>
+        </is>
+      </c>
+      <c r="F231" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G231" t="inlineStr">
+        <is>
+          <t>Neuronal</t>
+        </is>
+      </c>
+      <c r="H231" t="n">
+        <v>118</v>
+      </c>
+      <c r="I231" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>xenium_crc</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>fine</t>
+        </is>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>Tuft</t>
+        </is>
+      </c>
+      <c r="F232" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G232" t="inlineStr">
+        <is>
+          <t>Neuronal</t>
+        </is>
+      </c>
+      <c r="H232" t="n">
+        <v>25</v>
+      </c>
+      <c r="I232" t="n">
+        <v>9</v>
+      </c>
+      <c r="J232" t="inlineStr">
+        <is>
+          <t>Flex parent=Neuronal; pan-cancer v1 → Epithelial</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>xenium_crc</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>fine</t>
+        </is>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>Macrophage</t>
+        </is>
+      </c>
+      <c r="F233" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G233" t="inlineStr">
+        <is>
+          <t>Myeloid</t>
+        </is>
+      </c>
+      <c r="H233" t="n">
+        <v>1996</v>
+      </c>
+      <c r="I233" t="n">
+        <v>1998</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>xenium_crc</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>fine</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>Mast</t>
+        </is>
+      </c>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G234" t="inlineStr">
+        <is>
+          <t>Myeloid</t>
+        </is>
+      </c>
+      <c r="H234" t="n">
+        <v>211</v>
+      </c>
+      <c r="I234" t="n">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>xenium_crc</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>fine</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>Neutrophil</t>
+        </is>
+      </c>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G235" t="inlineStr">
+        <is>
+          <t>Myeloid</t>
+        </is>
+      </c>
+      <c r="H235" t="n">
+        <v>997</v>
+      </c>
+      <c r="I235" t="n">
+        <v>1727</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>xenium_crc</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>fine</t>
+        </is>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>Proliferating Macrophages</t>
+        </is>
+      </c>
+      <c r="F236" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G236" t="inlineStr">
+        <is>
+          <t>Myeloid</t>
+        </is>
+      </c>
+      <c r="H236" t="n">
+        <v>1433</v>
+      </c>
+      <c r="I236" t="n">
+        <v>1584</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>xenium_crc</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>fine</t>
+        </is>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>cDC I</t>
+        </is>
+      </c>
+      <c r="F237" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G237" t="inlineStr">
+        <is>
+          <t>Myeloid</t>
+        </is>
+      </c>
+      <c r="H237" t="n">
+        <v>204</v>
+      </c>
+      <c r="I237" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>xenium_crc</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>fine</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>mRegDC</t>
+        </is>
+      </c>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G238" t="inlineStr">
+        <is>
+          <t>Myeloid</t>
+        </is>
+      </c>
+      <c r="H238" t="n">
+        <v>320</v>
+      </c>
+      <c r="I238" t="n">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>xenium_crc</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>fine</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>pDC</t>
+        </is>
+      </c>
+      <c r="F239" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G239" t="inlineStr">
+        <is>
+          <t>Myeloid</t>
+        </is>
+      </c>
+      <c r="H239" t="n">
+        <v>24</v>
+      </c>
+      <c r="I239" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>xenium_crc</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>fine</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>CD4 T cell</t>
+        </is>
+      </c>
+      <c r="F240" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G240" t="inlineStr">
+        <is>
+          <t>T cells</t>
+        </is>
+      </c>
+      <c r="H240" t="n">
+        <v>4655</v>
+      </c>
+      <c r="I240" t="n">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>xenium_crc</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>fine</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>CD8 T cell</t>
+        </is>
+      </c>
+      <c r="F241" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G241" t="inlineStr">
+        <is>
+          <t>T cells</t>
+        </is>
+      </c>
+      <c r="H241" t="n">
+        <v>641</v>
+      </c>
+      <c r="I241" t="n">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>xenium_crc</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>fine</t>
+        </is>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>NK</t>
+        </is>
+      </c>
+      <c r="F242" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G242" t="inlineStr">
+        <is>
+          <t>T cells</t>
+        </is>
+      </c>
+      <c r="H242" t="n">
+        <v>16</v>
+      </c>
+      <c r="I242" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>xenium_crc</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>fine</t>
+        </is>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>Mature B</t>
+        </is>
+      </c>
+      <c r="F243" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G243" t="inlineStr">
+        <is>
+          <t>B cells</t>
+        </is>
+      </c>
+      <c r="H243" t="n">
+        <v>7704</v>
+      </c>
+      <c r="I243" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>xenium_crc</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>fine</t>
+        </is>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>Memory B</t>
+        </is>
+      </c>
+      <c r="F244" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G244" t="inlineStr">
+        <is>
+          <t>B cells</t>
+        </is>
+      </c>
+      <c r="H244" t="n">
+        <v>64</v>
+      </c>
+      <c r="I244" t="n">
+        <v>0</v>
+      </c>
+      <c r="J244" t="inlineStr">
+        <is>
+          <t>absent in P2 transferred singlets</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>xenium_crc</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>fine</t>
+        </is>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="F245" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G245" t="inlineStr">
+        <is>
+          <t>B cells</t>
+        </is>
+      </c>
+      <c r="H245" t="n">
+        <v>1198</v>
+      </c>
+      <c r="I245" t="n">
+        <v>3325</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>xenium_crc</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>fine</t>
+        </is>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>Proliferating Immune II</t>
+        </is>
+      </c>
+      <c r="F246" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G246" t="inlineStr">
+        <is>
+          <t>B cells</t>
+        </is>
+      </c>
+      <c r="H246" t="n">
+        <v>694</v>
+      </c>
+      <c r="I246" t="n">
+        <v>942</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>xenium_crc</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>fine</t>
+        </is>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>Endothelial</t>
+        </is>
+      </c>
+      <c r="F247" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G247" t="inlineStr">
+        <is>
+          <t>Endothelial</t>
+        </is>
+      </c>
+      <c r="H247" t="n">
+        <v>6189</v>
+      </c>
+      <c r="I247" t="n">
+        <v>4681</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>xenium_crc</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>fine</t>
+        </is>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>Lymphatic Endothelial</t>
+        </is>
+      </c>
+      <c r="F248" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G248" t="inlineStr">
+        <is>
+          <t>Endothelial</t>
+        </is>
+      </c>
+      <c r="H248" t="n">
+        <v>741</v>
+      </c>
+      <c r="I248" t="n">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>xenium_crc</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>fine</t>
+        </is>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>Unlabeled</t>
+        </is>
+      </c>
+      <c r="F249" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="J249" t="inlineStr">
+        <is>
+          <t>dropped at match; empty L1/L12</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>xenium_crc</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>intermediate</t>
+        </is>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>Tumor</t>
+        </is>
+      </c>
+      <c r="F250" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H250" t="n">
+        <v>81481</v>
+      </c>
+      <c r="I250" t="n">
+        <v>147751</v>
+      </c>
+      <c r="J250" t="inlineStr">
+        <is>
+          <t>Flex 2025 Level1 (9)</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>xenium_crc</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>intermediate</t>
+        </is>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>Intestinal Epithelial</t>
+        </is>
+      </c>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H251" t="n">
+        <v>22928</v>
+      </c>
+      <c r="I251" t="n">
+        <v>22205</v>
+      </c>
+      <c r="J251" t="inlineStr">
+        <is>
+          <t>Flex 2025 Level1 (9)</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>xenium_crc</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>intermediate</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>Fibroblast</t>
+        </is>
+      </c>
+      <c r="F252" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H252" t="n">
+        <v>20698</v>
+      </c>
+      <c r="I252" t="n">
+        <v>19863</v>
+      </c>
+      <c r="J252" t="inlineStr">
+        <is>
+          <t>Flex 2025 Level1 (9)</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>xenium_crc</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>intermediate</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>Smooth Muscle</t>
+        </is>
+      </c>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H253" t="n">
+        <v>2101</v>
+      </c>
+      <c r="I253" t="n">
+        <v>4346</v>
+      </c>
+      <c r="J253" t="inlineStr">
+        <is>
+          <t>Flex 2025 Level1 (9)</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>xenium_crc</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>intermediate</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>Myeloid</t>
+        </is>
+      </c>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H254" t="n">
+        <v>5185</v>
+      </c>
+      <c r="I254" t="n">
+        <v>5457</v>
+      </c>
+      <c r="J254" t="inlineStr">
+        <is>
+          <t>Flex 2025 Level1 (9)</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>xenium_crc</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>intermediate</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>T cells</t>
+        </is>
+      </c>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H255" t="n">
+        <v>5312</v>
+      </c>
+      <c r="I255" t="n">
+        <v>520</v>
+      </c>
+      <c r="J255" t="inlineStr">
+        <is>
+          <t>Flex 2025 Level1 (9)</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>xenium_crc</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>intermediate</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>B cells</t>
+        </is>
+      </c>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H256" t="n">
+        <v>9660</v>
+      </c>
+      <c r="I256" t="n">
+        <v>4281</v>
+      </c>
+      <c r="J256" t="inlineStr">
+        <is>
+          <t>Flex 2025 Level1 (9)</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>xenium_crc</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>intermediate</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>Endothelial</t>
+        </is>
+      </c>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H257" t="n">
+        <v>6930</v>
+      </c>
+      <c r="I257" t="n">
+        <v>5112</v>
+      </c>
+      <c r="J257" t="inlineStr">
+        <is>
+          <t>Flex 2025 Level1 (9)</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>xenium_crc</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>intermediate</t>
+        </is>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>Neuronal</t>
+        </is>
+      </c>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H258" t="n">
+        <v>465</v>
+      </c>
+      <c r="I258" t="n">
+        <v>244</v>
+      </c>
+      <c r="J258" t="inlineStr">
+        <is>
+          <t>Flex 2025 Level1 (9)</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>xenium_crc</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>coarse</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>Epithelial</t>
+        </is>
+      </c>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H259" t="n">
+        <v>104409</v>
+      </c>
+      <c r="I259" t="n">
+        <v>169956</v>
+      </c>
+      <c r="J259" t="inlineStr">
+        <is>
+          <t>Neuronal folded into Stromal</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>xenium_crc</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>coarse</t>
+        </is>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>Immune</t>
+        </is>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H260" t="n">
+        <v>20157</v>
+      </c>
+      <c r="I260" t="n">
+        <v>10258</v>
+      </c>
+      <c r="J260" t="inlineStr">
+        <is>
+          <t>Neuronal folded into Stromal</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>xenium_crc</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>coarse</t>
+        </is>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>Stromal</t>
+        </is>
+      </c>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H261" t="n">
+        <v>23264</v>
+      </c>
+      <c r="I261" t="n">
+        <v>24453</v>
+      </c>
+      <c r="J261" t="inlineStr">
+        <is>
+          <t>Neuronal folded into Stromal</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>xenium_crc</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>coarse</t>
+        </is>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>Endothelial</t>
+        </is>
+      </c>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H262" t="n">
+        <v>6930</v>
+      </c>
+      <c r="I262" t="n">
+        <v>5112</v>
+      </c>
+      <c r="J262" t="inlineStr">
+        <is>
+          <t>Neuronal folded into Stromal</t>
         </is>
       </c>
     </row>
@@ -11483,6 +14042,290 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="001F4E79"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="70" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Spatial_Data</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Cancer_Type</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Sample</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>HE_image</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>GT_cells_transferred</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>GT_cells_on_HE</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>StarDist_matched</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>StarDist_all</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>L2_all</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>L2_train</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>L12_train</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>L1_train</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Xenium</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>P1CRC</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>154760</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>154760</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>96858</v>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>1594379</v>
+      </c>
+      <c r="I2" s="3" t="n">
+        <v>38</v>
+      </c>
+      <c r="J2" s="3" t="n">
+        <v>38</v>
+      </c>
+      <c r="K2" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="L2" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>Sheet P1_CRC. Dominant Tumor II. StarDist present. HE OME ~0.274 µm/px.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Xenium</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>P2CRC</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>209779</v>
+      </c>
+      <c r="F3" s="5" t="n">
+        <v>209779</v>
+      </c>
+      <c r="G3" s="5" t="n">
+        <v>166503</v>
+      </c>
+      <c r="H3" s="5" t="n">
+        <v>1517884</v>
+      </c>
+      <c r="I3" s="5" t="n">
+        <v>36</v>
+      </c>
+      <c r="J3" s="5" t="n">
+        <v>38</v>
+      </c>
+      <c r="K3" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="L3" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="M3" s="4" t="inlineStr">
+        <is>
+          <t>Sheet P2_CRC. Dominant Tumor III. Missing Memory B and SM Stress Response in transferred singlets (hierarchy still 38).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Xenium</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>P5CRC</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="3" t="n"/>
+      <c r="I4" s="3" t="n"/>
+      <c r="J4" s="3" t="n"/>
+      <c r="K4" s="3" t="n"/>
+      <c r="L4" s="3" t="n"/>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>HE OME + he_imagealignment.csv present. No annotation sheet, Cases CSV, or StarDist yet. Xenium_P5_cell_info.csv has 1,029,090 cells.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Xenium</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>364539</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>364539</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>263361</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>3112263</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>39</v>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v>38</v>
+      </c>
+      <c r="K5" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="L5" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>Oliveira et al., Nat Genet 2025; GSE280318. Transferred RCTD singlet, not Xenium GT. L2_all 39 includes Unlabeled. P5 counted in HE_total only.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:M5"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -12255,7 +15098,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -12601,7 +15444,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -12912,185 +15755,4 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="55" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>coverslip</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>All_cores</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Annotated_cores</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Unlabeled_cores</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>GT_cells</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>L2_train</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="28" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>c009</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="n">
-        <v>160</v>
-      </c>
-      <c r="C2" s="3" t="n">
-        <v>160</v>
-      </c>
-      <c r="D2" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="3" t="n">
-        <v>11</v>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>GIST TMA</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="28" customHeight="1">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>c011</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="n">
-        <v>197</v>
-      </c>
-      <c r="C3" s="5" t="n">
-        <v>197</v>
-      </c>
-      <c r="D3" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E3" s="4" t="n"/>
-      <c r="F3" s="5" t="n">
-        <v>11</v>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>GIST TMA</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="28" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>c013</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="n">
-        <v>193</v>
-      </c>
-      <c r="C4" s="3" t="n">
-        <v>193</v>
-      </c>
-      <c r="D4" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E4" s="2" t="n"/>
-      <c r="F4" s="3" t="n">
-        <v>11</v>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>GIST TMA; demo Charvill-94_c013_v001_r001_reg002</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="28" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>All GIST</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="n">
-        <v>550</v>
-      </c>
-      <c r="C5" s="5" t="n">
-        <v>550</v>
-      </c>
-      <c r="D5" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E5" s="5" t="n">
-        <v>1785460</v>
-      </c>
-      <c r="F5" s="5" t="n">
-        <v>11</v>
-      </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>GT_cells from original overview (no Incomplete_Cases)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>L2 (11 train + Other): Epithelial cells, Fibroblasts, Stromal cells, Helper T cells, Tregs, T cells, Monocytes, Neutrophils, DCs, B cells, Endothelial cells, Other</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>L12/L1 same 6/4 structure as PDAC. Clinical recodes: site, size, mitotic, mutation, risk, primary, tma_block. StarDist: StarDist_Segment_gist/</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:G1"/>
-  <mergeCells count="2">
-    <mergeCell ref="A8:G8"/>
-    <mergeCell ref="A7:G7"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>